<commit_message>
Done Of the Concpet
</commit_message>
<xml_diff>
--- a/Sql/HD prob.xlsx
+++ b/Sql/HD prob.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ims-october-bkps\Sql\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8475405-EEE9-4716-94E6-332AFE4DA4E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{412AB534-9211-4A20-98F8-FC9818FD93DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23880" yWindow="630" windowWidth="20730" windowHeight="11040" tabRatio="692" firstSheet="7" activeTab="9" xr2:uid="{D32FFA46-9C2E-4324-9790-4976D8E4A0B4}"/>
+    <workbookView xWindow="23880" yWindow="630" windowWidth="20730" windowHeight="11040" tabRatio="692" firstSheet="7" activeTab="7" xr2:uid="{D32FFA46-9C2E-4324-9790-4976D8E4A0B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -20,9 +20,9 @@
     <sheet name="POS  and PAGE UPDATE" sheetId="7" state="hidden" r:id="rId5"/>
     <sheet name="Induction re-arrange" sheetId="13" state="hidden" r:id="rId6"/>
     <sheet name="re register" sheetId="12" state="hidden" r:id="rId7"/>
-    <sheet name="HD RESULT" sheetId="2" r:id="rId8"/>
+    <sheet name="Wanna Host Coreclty" sheetId="16" r:id="rId8"/>
     <sheet name="New ID Order Missing " sheetId="14" r:id="rId9"/>
-    <sheet name="Sheet3" sheetId="15" r:id="rId10"/>
+    <sheet name="HD RESULT another also" sheetId="2" r:id="rId10"/>
     <sheet name="Sheet2" sheetId="6" state="hidden" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="162">
   <si>
     <t>Re-sit</t>
   </si>
@@ -555,12 +555,54 @@
   <si>
     <t>transection_exams/save_assessment_document_send.php</t>
   </si>
+  <si>
+    <t xml:space="preserve">Updated into HOSTING </t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>view_details_of_exams_add_result.php</t>
+  </si>
+  <si>
+    <t>Updated on 14-09-2026</t>
+  </si>
+  <si>
+    <t>editAllocateProgram.php</t>
+  </si>
+  <si>
+    <t>added the compulsary checkbox here</t>
+  </si>
+  <si>
+    <t>single_views.php</t>
+  </si>
+  <si>
+    <t>Wanna Host</t>
+  </si>
+  <si>
+    <t>Hosted (Updated)</t>
+  </si>
+  <si>
+    <t>Date Hosted</t>
+  </si>
+  <si>
+    <t>15-09-2026 b1</t>
+  </si>
+  <si>
+    <t>15-09-2026 b2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exam_result_folder\save_results.php </t>
+  </si>
+  <si>
+    <t>24-08-2026 b1</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -655,8 +697,22 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -747,6 +803,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="31">
     <border>
@@ -1098,7 +1160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="156">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1259,16 +1321,19 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1289,9 +1354,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1307,11 +1369,125 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2376,26 +2552,26 @@
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="20"/>
-      <c r="C4" s="112" t="s">
+      <c r="C4" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="113"/>
-      <c r="E4" s="116" t="s">
+      <c r="D4" s="122"/>
+      <c r="E4" s="125" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="113" t="s">
+      <c r="F4" s="122" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="113"/>
+      <c r="G4" s="122"/>
       <c r="H4" s="7"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="21"/>
-      <c r="C5" s="114"/>
-      <c r="D5" s="115"/>
-      <c r="E5" s="117"/>
-      <c r="F5" s="115"/>
-      <c r="G5" s="115"/>
+      <c r="C5" s="123"/>
+      <c r="D5" s="124"/>
+      <c r="E5" s="126"/>
+      <c r="F5" s="124"/>
+      <c r="G5" s="124"/>
       <c r="H5" s="8"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
@@ -2817,26 +2993,121 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99CCEDAB-CE43-4A7E-B09A-9247E540F366}">
-  <dimension ref="D8:D9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46E2123E-1D13-46F0-9B4A-A5272E85634C}">
+  <dimension ref="A1:K18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="59.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="4" max="4" width="48" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="2.140625" customWidth="1"/>
+    <col min="10" max="10" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D8" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="9" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D9" t="s">
-        <v>147</v>
-      </c>
+    <row r="1" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C1" s="82"/>
+      <c r="D1" s="83"/>
+    </row>
+    <row r="2" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C2" s="84"/>
+      <c r="D2" s="85" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C3" s="84"/>
+      <c r="D3" s="85" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C4" s="84"/>
+      <c r="D4" s="85" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="84"/>
+      <c r="D5" s="85" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C6" s="84"/>
+      <c r="D6" s="85"/>
+      <c r="I6" s="116"/>
+      <c r="J6" s="111"/>
+      <c r="K6" s="112"/>
+    </row>
+    <row r="7" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C7" s="84"/>
+      <c r="D7" s="85"/>
+      <c r="I7" s="117"/>
+      <c r="J7" s="113" t="s">
+        <v>150</v>
+      </c>
+      <c r="K7" s="119" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="8" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="84"/>
+      <c r="D8" s="85" t="s">
+        <v>97</v>
+      </c>
+      <c r="I8" s="118"/>
+      <c r="J8" s="114"/>
+      <c r="K8" s="115"/>
+    </row>
+    <row r="9" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C9" s="84"/>
+      <c r="D9" s="85" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="10" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C10" s="84"/>
+      <c r="D10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="11" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="86"/>
+      <c r="D11" s="87"/>
+    </row>
+    <row r="15" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="D15" s="85"/>
+    </row>
+    <row r="16" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="D16" s="85"/>
+    </row>
+    <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="18" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="136" t="s">
+        <v>151</v>
+      </c>
+      <c r="B18" s="137"/>
+      <c r="C18" s="138"/>
+      <c r="D18" s="139" t="s">
+        <v>152</v>
+      </c>
+      <c r="E18" s="140" t="s">
+        <v>153</v>
+      </c>
+      <c r="F18" s="140"/>
+      <c r="G18" s="141"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="E18:G18"/>
+  </mergeCells>
+  <conditionalFormatting sqref="J7 D15:D1048576 D1:D13">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3089,10 +3360,10 @@
       </c>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="118" t="s">
+      <c r="B11" s="120" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="118"/>
+      <c r="C11" s="120"/>
       <c r="D11" s="31" t="s">
         <v>40</v>
       </c>
@@ -3112,10 +3383,10 @@
       </c>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="118" t="s">
+      <c r="B12" s="120" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="118"/>
+      <c r="C12" s="120"/>
       <c r="D12" s="31" t="s">
         <v>40</v>
       </c>
@@ -3448,17 +3719,17 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C3" s="119" t="s">
+      <c r="C3" s="127" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="119"/>
-      <c r="E3" s="119"/>
-      <c r="L3" s="119" t="s">
+      <c r="D3" s="127"/>
+      <c r="E3" s="127"/>
+      <c r="L3" s="127" t="s">
         <v>92</v>
       </c>
-      <c r="M3" s="119"/>
-      <c r="N3" s="119"/>
-      <c r="O3" s="119"/>
+      <c r="M3" s="127"/>
+      <c r="N3" s="127"/>
+      <c r="O3" s="127"/>
       <c r="Q3" s="76" t="s">
         <v>94</v>
       </c>
@@ -4236,7 +4507,7 @@
     <mergeCell ref="L3:O3"/>
   </mergeCells>
   <conditionalFormatting sqref="K15:O17 A15:J16 B17:J17 B4:O14 B18:O38">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -4275,11 +4546,11 @@
       <c r="E3" s="81">
         <v>46121</v>
       </c>
-      <c r="H3" s="120" t="s">
+      <c r="H3" s="128" t="s">
         <v>109</v>
       </c>
-      <c r="I3" s="121"/>
-      <c r="J3" s="122"/>
+      <c r="I3" s="129"/>
+      <c r="J3" s="130"/>
     </row>
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="84"/>
@@ -4581,7 +4852,7 @@
     <sortCondition ref="C1:C27"/>
   </sortState>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -4611,15 +4882,15 @@
       <c r="C3" s="83" t="s">
         <v>116</v>
       </c>
-      <c r="F3" s="123" t="s">
+      <c r="F3" s="131" t="s">
         <v>120</v>
       </c>
-      <c r="G3" s="123"/>
-      <c r="H3" s="123"/>
-      <c r="I3" s="123"/>
-      <c r="J3" s="123"/>
-      <c r="K3" s="123"/>
-      <c r="L3" s="123"/>
+      <c r="G3" s="131"/>
+      <c r="H3" s="131"/>
+      <c r="I3" s="131"/>
+      <c r="J3" s="131"/>
+      <c r="K3" s="131"/>
+      <c r="L3" s="131"/>
     </row>
     <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="101"/>
@@ -4739,46 +5010,1085 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46E2123E-1D13-46F0-9B4A-A5272E85634C}">
-  <dimension ref="D2:D9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68875BD9-58CC-4CDF-864D-5941A765C906}">
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+  </sheetPr>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="48" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.140625" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="2.7109375" customWidth="1"/>
+    <col min="6" max="6" width="2.85546875" customWidth="1"/>
+    <col min="7" max="7" width="4" customWidth="1"/>
+    <col min="8" max="8" width="2.42578125" customWidth="1"/>
+    <col min="9" max="9" width="56.140625" customWidth="1"/>
+    <col min="10" max="10" width="9.140625" customWidth="1"/>
+    <col min="11" max="11" width="19.85546875" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D2" t="s">
+    <row r="1" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="143" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" s="144"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="145"/>
+      <c r="G1" s="146" t="s">
+        <v>156</v>
+      </c>
+      <c r="H1" s="147"/>
+      <c r="I1" s="147"/>
+      <c r="J1" s="147"/>
+      <c r="K1" s="147"/>
+      <c r="L1" s="147"/>
+      <c r="M1" s="147"/>
+      <c r="N1" s="147"/>
+      <c r="O1" s="147"/>
+      <c r="P1" s="147"/>
+      <c r="Q1" s="148"/>
+    </row>
+    <row r="2" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="149"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
+      <c r="E2" s="150"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="152"/>
+      <c r="H2" s="153"/>
+      <c r="I2" s="153"/>
+      <c r="J2" s="153"/>
+      <c r="K2" s="153"/>
+      <c r="L2" s="153"/>
+      <c r="M2" s="153"/>
+      <c r="N2" s="153"/>
+      <c r="O2" s="153"/>
+      <c r="P2" s="153"/>
+      <c r="Q2" s="154"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="84"/>
+      <c r="B3" s="142"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="142"/>
+      <c r="F3" s="85"/>
+      <c r="G3" s="84"/>
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142" t="s">
+        <v>157</v>
+      </c>
+      <c r="L3" s="142"/>
+      <c r="M3" s="142"/>
+      <c r="N3" s="142"/>
+      <c r="O3" s="142"/>
+      <c r="P3" s="142"/>
+      <c r="Q3" s="85"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="84"/>
+      <c r="B4" s="142" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
+      <c r="C4" s="142"/>
+      <c r="D4" s="142"/>
+      <c r="E4" s="142"/>
+      <c r="F4" s="85"/>
+      <c r="G4" s="84" t="s">
+        <v>137</v>
+      </c>
+      <c r="H4" s="142"/>
+      <c r="I4" s="155" t="s">
+        <v>144</v>
+      </c>
+      <c r="J4" s="142"/>
+      <c r="K4" s="142"/>
+      <c r="L4" s="142"/>
+      <c r="M4" s="142"/>
+      <c r="N4" s="142"/>
+      <c r="O4" s="142"/>
+      <c r="P4" s="142"/>
+      <c r="Q4" s="85"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="84"/>
+      <c r="B5" s="142" t="s">
+        <v>160</v>
+      </c>
+      <c r="C5" s="142" t="s">
+        <v>161</v>
+      </c>
+      <c r="D5" s="142"/>
+      <c r="E5" s="142"/>
+      <c r="F5" s="85"/>
+      <c r="G5" s="84" t="s">
+        <v>137</v>
+      </c>
+      <c r="H5" s="142"/>
+      <c r="I5" s="155" t="s">
+        <v>146</v>
+      </c>
+      <c r="J5" s="142"/>
+      <c r="K5" s="142"/>
+      <c r="L5" s="142"/>
+      <c r="M5" s="142"/>
+      <c r="N5" s="142"/>
+      <c r="O5" s="142"/>
+      <c r="P5" s="142"/>
+      <c r="Q5" s="85"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" s="84"/>
+      <c r="B6" s="142" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
+      <c r="C6" s="142"/>
+      <c r="D6" s="142"/>
+      <c r="E6" s="142"/>
+      <c r="F6" s="85"/>
+      <c r="G6" s="84" t="s">
+        <v>137</v>
+      </c>
+      <c r="H6" s="142"/>
+      <c r="I6" s="155" t="s">
+        <v>147</v>
+      </c>
+      <c r="J6" s="142"/>
+      <c r="K6" s="142"/>
+      <c r="L6" s="142"/>
+      <c r="M6" s="142"/>
+      <c r="N6" s="142"/>
+      <c r="O6" s="142"/>
+      <c r="P6" s="142"/>
+      <c r="Q6" s="85"/>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="84"/>
+      <c r="B7" s="142" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D8" t="s">
+      <c r="C7" s="142"/>
+      <c r="D7" s="142"/>
+      <c r="E7" s="142"/>
+      <c r="F7" s="85"/>
+      <c r="G7" s="84"/>
+      <c r="H7" s="142"/>
+      <c r="I7" s="142"/>
+      <c r="J7" s="142"/>
+      <c r="K7" s="142"/>
+      <c r="L7" s="142"/>
+      <c r="M7" s="142"/>
+      <c r="N7" s="142"/>
+      <c r="O7" s="142"/>
+      <c r="P7" s="142"/>
+      <c r="Q7" s="85"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="84"/>
+      <c r="B8" s="142"/>
+      <c r="C8" s="142"/>
+      <c r="D8" s="142"/>
+      <c r="E8" s="142"/>
+      <c r="F8" s="85"/>
+      <c r="G8" s="84" t="s">
+        <v>137</v>
+      </c>
+      <c r="H8" s="142"/>
+      <c r="I8" s="142" t="s">
+        <v>63</v>
+      </c>
+      <c r="J8" s="142"/>
+      <c r="K8" s="142" t="s">
+        <v>158</v>
+      </c>
+      <c r="L8" s="142"/>
+      <c r="M8" s="142"/>
+      <c r="N8" s="142"/>
+      <c r="O8" s="142"/>
+      <c r="P8" s="142"/>
+      <c r="Q8" s="85"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="84"/>
+      <c r="B9" s="142" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="9" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D9" t="s">
+      <c r="C9" s="142"/>
+      <c r="D9" s="142"/>
+      <c r="E9" s="142"/>
+      <c r="F9" s="85"/>
+      <c r="G9" s="84" t="s">
+        <v>137</v>
+      </c>
+      <c r="H9" s="142"/>
+      <c r="I9" s="142" t="s">
+        <v>124</v>
+      </c>
+      <c r="J9" s="142"/>
+      <c r="K9" s="142" t="s">
+        <v>159</v>
+      </c>
+      <c r="L9" s="142"/>
+      <c r="M9" s="142"/>
+      <c r="N9" s="142"/>
+      <c r="O9" s="142"/>
+      <c r="P9" s="142"/>
+      <c r="Q9" s="85"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="84"/>
+      <c r="B10" s="142" t="s">
         <v>98</v>
       </c>
+      <c r="C10" s="142"/>
+      <c r="D10" s="142"/>
+      <c r="E10" s="142"/>
+      <c r="F10" s="85"/>
+      <c r="G10" s="84"/>
+      <c r="H10" s="142"/>
+      <c r="I10" s="142"/>
+      <c r="J10" s="142"/>
+      <c r="K10" s="142"/>
+      <c r="L10" s="142"/>
+      <c r="M10" s="142"/>
+      <c r="N10" s="142"/>
+      <c r="O10" s="142"/>
+      <c r="P10" s="142"/>
+      <c r="Q10" s="85"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" s="84"/>
+      <c r="B11" s="142" t="s">
+        <v>154</v>
+      </c>
+      <c r="C11" s="142"/>
+      <c r="D11" s="142"/>
+      <c r="E11" s="142"/>
+      <c r="F11" s="85"/>
+      <c r="G11" s="84"/>
+      <c r="H11" s="142"/>
+      <c r="I11" s="142"/>
+      <c r="J11" s="142"/>
+      <c r="K11" s="142"/>
+      <c r="L11" s="142"/>
+      <c r="M11" s="142"/>
+      <c r="N11" s="142"/>
+      <c r="O11" s="142"/>
+      <c r="P11" s="142"/>
+      <c r="Q11" s="85"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" s="84"/>
+      <c r="B12" s="142"/>
+      <c r="C12" s="142"/>
+      <c r="D12" s="142"/>
+      <c r="E12" s="142"/>
+      <c r="F12" s="85"/>
+      <c r="G12" s="84"/>
+      <c r="H12" s="142"/>
+      <c r="I12" s="142"/>
+      <c r="J12" s="142"/>
+      <c r="K12" s="142"/>
+      <c r="L12" s="142"/>
+      <c r="M12" s="142"/>
+      <c r="N12" s="142"/>
+      <c r="O12" s="142"/>
+      <c r="P12" s="142"/>
+      <c r="Q12" s="85"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13" s="84"/>
+      <c r="C13" s="142"/>
+      <c r="D13" s="142"/>
+      <c r="E13" s="142"/>
+      <c r="F13" s="85"/>
+      <c r="G13" s="84"/>
+      <c r="H13" s="142"/>
+      <c r="I13" s="142"/>
+      <c r="J13" s="142"/>
+      <c r="K13" s="142"/>
+      <c r="L13" s="142"/>
+      <c r="M13" s="142"/>
+      <c r="N13" s="142"/>
+      <c r="O13" s="142"/>
+      <c r="P13" s="142"/>
+      <c r="Q13" s="85"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" s="84"/>
+      <c r="C14" s="142"/>
+      <c r="D14" s="142"/>
+      <c r="E14" s="142"/>
+      <c r="F14" s="85"/>
+      <c r="G14" s="84"/>
+      <c r="H14" s="142"/>
+      <c r="I14" s="142"/>
+      <c r="J14" s="142"/>
+      <c r="K14" s="142"/>
+      <c r="L14" s="142"/>
+      <c r="M14" s="142"/>
+      <c r="N14" s="142"/>
+      <c r="O14" s="142"/>
+      <c r="P14" s="142"/>
+      <c r="Q14" s="85"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15" s="84"/>
+      <c r="B15" s="142"/>
+      <c r="C15" s="142"/>
+      <c r="D15" s="142"/>
+      <c r="E15" s="142"/>
+      <c r="F15" s="85"/>
+      <c r="G15" s="84"/>
+      <c r="H15" s="142"/>
+      <c r="I15" s="142"/>
+      <c r="J15" s="142"/>
+      <c r="K15" s="142"/>
+      <c r="L15" s="142"/>
+      <c r="M15" s="142"/>
+      <c r="N15" s="142"/>
+      <c r="O15" s="142"/>
+      <c r="P15" s="142"/>
+      <c r="Q15" s="85"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" s="84"/>
+      <c r="B16" s="142"/>
+      <c r="C16" s="142"/>
+      <c r="D16" s="142"/>
+      <c r="E16" s="142"/>
+      <c r="F16" s="85"/>
+      <c r="G16" s="84"/>
+      <c r="H16" s="142"/>
+      <c r="I16" s="142"/>
+      <c r="J16" s="142"/>
+      <c r="K16" s="142"/>
+      <c r="L16" s="142"/>
+      <c r="M16" s="142"/>
+      <c r="N16" s="142"/>
+      <c r="O16" s="142"/>
+      <c r="P16" s="142"/>
+      <c r="Q16" s="85"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A17" s="84"/>
+      <c r="B17" s="142"/>
+      <c r="C17" s="142"/>
+      <c r="D17" s="142"/>
+      <c r="E17" s="142"/>
+      <c r="F17" s="85"/>
+      <c r="G17" s="84"/>
+      <c r="H17" s="142"/>
+      <c r="I17" s="142"/>
+      <c r="J17" s="142"/>
+      <c r="K17" s="142"/>
+      <c r="L17" s="142"/>
+      <c r="M17" s="142"/>
+      <c r="N17" s="142"/>
+      <c r="O17" s="142"/>
+      <c r="P17" s="142"/>
+      <c r="Q17" s="85"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A18" s="84"/>
+      <c r="B18" s="142"/>
+      <c r="C18" s="142"/>
+      <c r="D18" s="142"/>
+      <c r="E18" s="142"/>
+      <c r="F18" s="85"/>
+      <c r="G18" s="84"/>
+      <c r="H18" s="142"/>
+      <c r="I18" s="142"/>
+      <c r="J18" s="142"/>
+      <c r="K18" s="142"/>
+      <c r="L18" s="142"/>
+      <c r="M18" s="142"/>
+      <c r="N18" s="142"/>
+      <c r="O18" s="142"/>
+      <c r="P18" s="142"/>
+      <c r="Q18" s="85"/>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A19" s="84"/>
+      <c r="B19" s="142"/>
+      <c r="C19" s="142"/>
+      <c r="D19" s="142"/>
+      <c r="E19" s="142"/>
+      <c r="F19" s="85"/>
+      <c r="G19" s="84"/>
+      <c r="H19" s="142"/>
+      <c r="I19" s="142"/>
+      <c r="J19" s="142"/>
+      <c r="K19" s="142"/>
+      <c r="L19" s="142"/>
+      <c r="M19" s="142"/>
+      <c r="N19" s="142"/>
+      <c r="O19" s="142"/>
+      <c r="P19" s="142"/>
+      <c r="Q19" s="85"/>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A20" s="84"/>
+      <c r="B20" s="142"/>
+      <c r="C20" s="142"/>
+      <c r="D20" s="142"/>
+      <c r="E20" s="142"/>
+      <c r="F20" s="85"/>
+      <c r="G20" s="84"/>
+      <c r="H20" s="142"/>
+      <c r="I20" s="142"/>
+      <c r="J20" s="142"/>
+      <c r="K20" s="142"/>
+      <c r="L20" s="142"/>
+      <c r="M20" s="142"/>
+      <c r="N20" s="142"/>
+      <c r="O20" s="142"/>
+      <c r="P20" s="142"/>
+      <c r="Q20" s="85"/>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A21" s="84"/>
+      <c r="B21" s="142"/>
+      <c r="C21" s="142"/>
+      <c r="D21" s="142"/>
+      <c r="E21" s="142"/>
+      <c r="F21" s="85"/>
+      <c r="G21" s="84"/>
+      <c r="H21" s="142"/>
+      <c r="I21" s="142"/>
+      <c r="J21" s="142"/>
+      <c r="K21" s="142"/>
+      <c r="L21" s="142"/>
+      <c r="M21" s="142"/>
+      <c r="N21" s="142"/>
+      <c r="O21" s="142"/>
+      <c r="P21" s="142"/>
+      <c r="Q21" s="85"/>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A22" s="84"/>
+      <c r="B22" s="142"/>
+      <c r="C22" s="142"/>
+      <c r="D22" s="142"/>
+      <c r="E22" s="142"/>
+      <c r="F22" s="85"/>
+      <c r="G22" s="84"/>
+      <c r="H22" s="142"/>
+      <c r="I22" s="142"/>
+      <c r="J22" s="142"/>
+      <c r="K22" s="142"/>
+      <c r="L22" s="142"/>
+      <c r="M22" s="142"/>
+      <c r="N22" s="142"/>
+      <c r="O22" s="142"/>
+      <c r="P22" s="142"/>
+      <c r="Q22" s="85"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A23" s="84"/>
+      <c r="B23" s="142"/>
+      <c r="C23" s="142"/>
+      <c r="D23" s="142"/>
+      <c r="E23" s="142"/>
+      <c r="F23" s="85"/>
+      <c r="G23" s="84"/>
+      <c r="H23" s="142"/>
+      <c r="I23" s="142"/>
+      <c r="J23" s="142"/>
+      <c r="K23" s="142"/>
+      <c r="L23" s="142"/>
+      <c r="M23" s="142"/>
+      <c r="N23" s="142"/>
+      <c r="O23" s="142"/>
+      <c r="P23" s="142"/>
+      <c r="Q23" s="85"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A24" s="84"/>
+      <c r="B24" s="142"/>
+      <c r="C24" s="142"/>
+      <c r="D24" s="142"/>
+      <c r="E24" s="142"/>
+      <c r="F24" s="85"/>
+      <c r="G24" s="84"/>
+      <c r="H24" s="142"/>
+      <c r="I24" s="142"/>
+      <c r="J24" s="142"/>
+      <c r="K24" s="142"/>
+      <c r="L24" s="142"/>
+      <c r="M24" s="142"/>
+      <c r="N24" s="142"/>
+      <c r="O24" s="142"/>
+      <c r="P24" s="142"/>
+      <c r="Q24" s="85"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A25" s="84"/>
+      <c r="B25" s="142"/>
+      <c r="C25" s="142"/>
+      <c r="D25" s="142"/>
+      <c r="E25" s="142"/>
+      <c r="F25" s="85"/>
+      <c r="G25" s="84"/>
+      <c r="H25" s="142"/>
+      <c r="I25" s="142"/>
+      <c r="J25" s="142"/>
+      <c r="K25" s="142"/>
+      <c r="L25" s="142"/>
+      <c r="M25" s="142"/>
+      <c r="N25" s="142"/>
+      <c r="O25" s="142"/>
+      <c r="P25" s="142"/>
+      <c r="Q25" s="85"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A26" s="84"/>
+      <c r="B26" s="142"/>
+      <c r="C26" s="142"/>
+      <c r="D26" s="142"/>
+      <c r="E26" s="142"/>
+      <c r="F26" s="85"/>
+      <c r="G26" s="84"/>
+      <c r="H26" s="142"/>
+      <c r="I26" s="142"/>
+      <c r="J26" s="142"/>
+      <c r="K26" s="142"/>
+      <c r="L26" s="142"/>
+      <c r="M26" s="142"/>
+      <c r="N26" s="142"/>
+      <c r="O26" s="142"/>
+      <c r="P26" s="142"/>
+      <c r="Q26" s="85"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A27" s="84"/>
+      <c r="B27" s="142"/>
+      <c r="C27" s="142"/>
+      <c r="D27" s="142"/>
+      <c r="E27" s="142"/>
+      <c r="F27" s="85"/>
+      <c r="G27" s="84"/>
+      <c r="H27" s="142"/>
+      <c r="I27" s="142"/>
+      <c r="J27" s="142"/>
+      <c r="K27" s="142"/>
+      <c r="L27" s="142"/>
+      <c r="M27" s="142"/>
+      <c r="N27" s="142"/>
+      <c r="O27" s="142"/>
+      <c r="P27" s="142"/>
+      <c r="Q27" s="85"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A28" s="84"/>
+      <c r="B28" s="142"/>
+      <c r="C28" s="142"/>
+      <c r="D28" s="142"/>
+      <c r="E28" s="142"/>
+      <c r="F28" s="85"/>
+      <c r="G28" s="84"/>
+      <c r="H28" s="142"/>
+      <c r="I28" s="142"/>
+      <c r="J28" s="142"/>
+      <c r="K28" s="142"/>
+      <c r="L28" s="142"/>
+      <c r="M28" s="142"/>
+      <c r="N28" s="142"/>
+      <c r="O28" s="142"/>
+      <c r="P28" s="142"/>
+      <c r="Q28" s="85"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A29" s="84"/>
+      <c r="B29" s="142"/>
+      <c r="C29" s="142"/>
+      <c r="D29" s="142"/>
+      <c r="E29" s="142"/>
+      <c r="F29" s="85"/>
+      <c r="G29" s="84"/>
+      <c r="H29" s="142"/>
+      <c r="I29" s="142"/>
+      <c r="J29" s="142"/>
+      <c r="K29" s="142"/>
+      <c r="L29" s="142"/>
+      <c r="M29" s="142"/>
+      <c r="N29" s="142"/>
+      <c r="O29" s="142"/>
+      <c r="P29" s="142"/>
+      <c r="Q29" s="85"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A30" s="84"/>
+      <c r="B30" s="142"/>
+      <c r="C30" s="142"/>
+      <c r="D30" s="142"/>
+      <c r="E30" s="142"/>
+      <c r="F30" s="85"/>
+      <c r="G30" s="84"/>
+      <c r="H30" s="142"/>
+      <c r="I30" s="142"/>
+      <c r="J30" s="142"/>
+      <c r="K30" s="142"/>
+      <c r="L30" s="142"/>
+      <c r="M30" s="142"/>
+      <c r="N30" s="142"/>
+      <c r="O30" s="142"/>
+      <c r="P30" s="142"/>
+      <c r="Q30" s="85"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A31" s="84"/>
+      <c r="B31" s="142"/>
+      <c r="C31" s="142"/>
+      <c r="D31" s="142"/>
+      <c r="E31" s="142"/>
+      <c r="F31" s="85"/>
+      <c r="G31" s="84"/>
+      <c r="H31" s="142"/>
+      <c r="I31" s="142"/>
+      <c r="J31" s="142"/>
+      <c r="K31" s="142"/>
+      <c r="L31" s="142"/>
+      <c r="M31" s="142"/>
+      <c r="N31" s="142"/>
+      <c r="O31" s="142"/>
+      <c r="P31" s="142"/>
+      <c r="Q31" s="85"/>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A32" s="84"/>
+      <c r="B32" s="142"/>
+      <c r="C32" s="142"/>
+      <c r="D32" s="142"/>
+      <c r="E32" s="142"/>
+      <c r="F32" s="85"/>
+      <c r="G32" s="84"/>
+      <c r="H32" s="142"/>
+      <c r="I32" s="142"/>
+      <c r="J32" s="142"/>
+      <c r="K32" s="142"/>
+      <c r="L32" s="142"/>
+      <c r="M32" s="142"/>
+      <c r="N32" s="142"/>
+      <c r="O32" s="142"/>
+      <c r="P32" s="142"/>
+      <c r="Q32" s="85"/>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A33" s="84"/>
+      <c r="B33" s="142"/>
+      <c r="C33" s="142"/>
+      <c r="D33" s="142"/>
+      <c r="E33" s="142"/>
+      <c r="F33" s="85"/>
+      <c r="G33" s="84"/>
+      <c r="H33" s="142"/>
+      <c r="I33" s="142"/>
+      <c r="J33" s="142"/>
+      <c r="K33" s="142"/>
+      <c r="L33" s="142"/>
+      <c r="M33" s="142"/>
+      <c r="N33" s="142"/>
+      <c r="O33" s="142"/>
+      <c r="P33" s="142"/>
+      <c r="Q33" s="85"/>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A34" s="84"/>
+      <c r="B34" s="142"/>
+      <c r="C34" s="142"/>
+      <c r="D34" s="142"/>
+      <c r="E34" s="142"/>
+      <c r="F34" s="85"/>
+      <c r="G34" s="84"/>
+      <c r="H34" s="142"/>
+      <c r="I34" s="142"/>
+      <c r="J34" s="142"/>
+      <c r="K34" s="142"/>
+      <c r="L34" s="142"/>
+      <c r="M34" s="142"/>
+      <c r="N34" s="142"/>
+      <c r="O34" s="142"/>
+      <c r="P34" s="142"/>
+      <c r="Q34" s="85"/>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A35" s="84"/>
+      <c r="B35" s="142"/>
+      <c r="C35" s="142"/>
+      <c r="D35" s="142"/>
+      <c r="E35" s="142"/>
+      <c r="F35" s="85"/>
+      <c r="G35" s="84"/>
+      <c r="H35" s="142"/>
+      <c r="I35" s="142"/>
+      <c r="J35" s="142"/>
+      <c r="K35" s="142"/>
+      <c r="L35" s="142"/>
+      <c r="M35" s="142"/>
+      <c r="N35" s="142"/>
+      <c r="O35" s="142"/>
+      <c r="P35" s="142"/>
+      <c r="Q35" s="85"/>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A36" s="84"/>
+      <c r="B36" s="142"/>
+      <c r="C36" s="142"/>
+      <c r="D36" s="142"/>
+      <c r="E36" s="142"/>
+      <c r="F36" s="85"/>
+      <c r="G36" s="84"/>
+      <c r="H36" s="142"/>
+      <c r="I36" s="142"/>
+      <c r="J36" s="142"/>
+      <c r="K36" s="142"/>
+      <c r="L36" s="142"/>
+      <c r="M36" s="142"/>
+      <c r="N36" s="142"/>
+      <c r="O36" s="142"/>
+      <c r="P36" s="142"/>
+      <c r="Q36" s="85"/>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A37" s="84"/>
+      <c r="B37" s="142"/>
+      <c r="C37" s="142"/>
+      <c r="D37" s="142"/>
+      <c r="E37" s="142"/>
+      <c r="F37" s="85"/>
+      <c r="G37" s="84"/>
+      <c r="H37" s="142"/>
+      <c r="I37" s="142"/>
+      <c r="J37" s="142"/>
+      <c r="K37" s="142"/>
+      <c r="L37" s="142"/>
+      <c r="M37" s="142"/>
+      <c r="N37" s="142"/>
+      <c r="O37" s="142"/>
+      <c r="P37" s="142"/>
+      <c r="Q37" s="85"/>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A38" s="84"/>
+      <c r="B38" s="142"/>
+      <c r="C38" s="142"/>
+      <c r="D38" s="142"/>
+      <c r="E38" s="142"/>
+      <c r="F38" s="85"/>
+      <c r="G38" s="84"/>
+      <c r="H38" s="142"/>
+      <c r="I38" s="142"/>
+      <c r="J38" s="142"/>
+      <c r="K38" s="142"/>
+      <c r="L38" s="142"/>
+      <c r="M38" s="142"/>
+      <c r="N38" s="142"/>
+      <c r="O38" s="142"/>
+      <c r="P38" s="142"/>
+      <c r="Q38" s="85"/>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A39" s="84"/>
+      <c r="B39" s="142"/>
+      <c r="C39" s="142"/>
+      <c r="D39" s="142"/>
+      <c r="E39" s="142"/>
+      <c r="F39" s="85"/>
+      <c r="G39" s="84"/>
+      <c r="H39" s="142"/>
+      <c r="I39" s="142"/>
+      <c r="J39" s="142"/>
+      <c r="K39" s="142"/>
+      <c r="L39" s="142"/>
+      <c r="M39" s="142"/>
+      <c r="N39" s="142"/>
+      <c r="O39" s="142"/>
+      <c r="P39" s="142"/>
+      <c r="Q39" s="85"/>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A40" s="84"/>
+      <c r="B40" s="142"/>
+      <c r="C40" s="142"/>
+      <c r="D40" s="142"/>
+      <c r="E40" s="142"/>
+      <c r="F40" s="85"/>
+      <c r="G40" s="84"/>
+      <c r="H40" s="142"/>
+      <c r="I40" s="142"/>
+      <c r="J40" s="142"/>
+      <c r="K40" s="142"/>
+      <c r="L40" s="142"/>
+      <c r="M40" s="142"/>
+      <c r="N40" s="142"/>
+      <c r="O40" s="142"/>
+      <c r="P40" s="142"/>
+      <c r="Q40" s="85"/>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A41" s="84"/>
+      <c r="B41" s="142"/>
+      <c r="C41" s="142"/>
+      <c r="D41" s="142"/>
+      <c r="E41" s="142"/>
+      <c r="F41" s="85"/>
+      <c r="G41" s="84"/>
+      <c r="H41" s="142"/>
+      <c r="I41" s="142"/>
+      <c r="J41" s="142"/>
+      <c r="K41" s="142"/>
+      <c r="L41" s="142"/>
+      <c r="M41" s="142"/>
+      <c r="N41" s="142"/>
+      <c r="O41" s="142"/>
+      <c r="P41" s="142"/>
+      <c r="Q41" s="85"/>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A42" s="84"/>
+      <c r="B42" s="142"/>
+      <c r="C42" s="142"/>
+      <c r="D42" s="142"/>
+      <c r="E42" s="142"/>
+      <c r="F42" s="85"/>
+      <c r="G42" s="84"/>
+      <c r="H42" s="142"/>
+      <c r="I42" s="142"/>
+      <c r="J42" s="142"/>
+      <c r="K42" s="142"/>
+      <c r="L42" s="142"/>
+      <c r="M42" s="142"/>
+      <c r="N42" s="142"/>
+      <c r="O42" s="142"/>
+      <c r="P42" s="142"/>
+      <c r="Q42" s="85"/>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A43" s="84"/>
+      <c r="B43" s="142"/>
+      <c r="C43" s="142"/>
+      <c r="D43" s="142"/>
+      <c r="E43" s="142"/>
+      <c r="F43" s="85"/>
+      <c r="G43" s="84"/>
+      <c r="H43" s="142"/>
+      <c r="I43" s="142"/>
+      <c r="J43" s="142"/>
+      <c r="K43" s="142"/>
+      <c r="L43" s="142"/>
+      <c r="M43" s="142"/>
+      <c r="N43" s="142"/>
+      <c r="O43" s="142"/>
+      <c r="P43" s="142"/>
+      <c r="Q43" s="85"/>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A44" s="84"/>
+      <c r="B44" s="142"/>
+      <c r="C44" s="142"/>
+      <c r="D44" s="142"/>
+      <c r="E44" s="142"/>
+      <c r="F44" s="85"/>
+      <c r="G44" s="84"/>
+      <c r="H44" s="142"/>
+      <c r="I44" s="142"/>
+      <c r="J44" s="142"/>
+      <c r="K44" s="142"/>
+      <c r="L44" s="142"/>
+      <c r="M44" s="142"/>
+      <c r="N44" s="142"/>
+      <c r="O44" s="142"/>
+      <c r="P44" s="142"/>
+      <c r="Q44" s="85"/>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A45" s="84"/>
+      <c r="B45" s="142"/>
+      <c r="C45" s="142"/>
+      <c r="D45" s="142"/>
+      <c r="E45" s="142"/>
+      <c r="F45" s="85"/>
+      <c r="G45" s="84"/>
+      <c r="H45" s="142"/>
+      <c r="I45" s="142"/>
+      <c r="J45" s="142"/>
+      <c r="K45" s="142"/>
+      <c r="L45" s="142"/>
+      <c r="M45" s="142"/>
+      <c r="N45" s="142"/>
+      <c r="O45" s="142"/>
+      <c r="P45" s="142"/>
+      <c r="Q45" s="85"/>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A46" s="84"/>
+      <c r="B46" s="142"/>
+      <c r="C46" s="142"/>
+      <c r="D46" s="142"/>
+      <c r="E46" s="142"/>
+      <c r="F46" s="85"/>
+      <c r="G46" s="84"/>
+      <c r="H46" s="142"/>
+      <c r="I46" s="142"/>
+      <c r="J46" s="142"/>
+      <c r="K46" s="142"/>
+      <c r="L46" s="142"/>
+      <c r="M46" s="142"/>
+      <c r="N46" s="142"/>
+      <c r="O46" s="142"/>
+      <c r="P46" s="142"/>
+      <c r="Q46" s="85"/>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A47" s="84"/>
+      <c r="B47" s="142"/>
+      <c r="C47" s="142"/>
+      <c r="D47" s="142"/>
+      <c r="E47" s="142"/>
+      <c r="F47" s="85"/>
+      <c r="G47" s="84"/>
+      <c r="H47" s="142"/>
+      <c r="I47" s="142"/>
+      <c r="J47" s="142"/>
+      <c r="K47" s="142"/>
+      <c r="L47" s="142"/>
+      <c r="M47" s="142"/>
+      <c r="N47" s="142"/>
+      <c r="O47" s="142"/>
+      <c r="P47" s="142"/>
+      <c r="Q47" s="85"/>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A48" s="84"/>
+      <c r="B48" s="142"/>
+      <c r="C48" s="142"/>
+      <c r="D48" s="142"/>
+      <c r="E48" s="142"/>
+      <c r="F48" s="85"/>
+      <c r="G48" s="84"/>
+      <c r="H48" s="142"/>
+      <c r="I48" s="142"/>
+      <c r="J48" s="142"/>
+      <c r="K48" s="142"/>
+      <c r="L48" s="142"/>
+      <c r="M48" s="142"/>
+      <c r="N48" s="142"/>
+      <c r="O48" s="142"/>
+      <c r="P48" s="142"/>
+      <c r="Q48" s="85"/>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A49" s="84"/>
+      <c r="B49" s="142"/>
+      <c r="C49" s="142"/>
+      <c r="D49" s="142"/>
+      <c r="E49" s="142"/>
+      <c r="F49" s="85"/>
+      <c r="G49" s="84"/>
+      <c r="H49" s="142"/>
+      <c r="I49" s="142"/>
+      <c r="J49" s="142"/>
+      <c r="K49" s="142"/>
+      <c r="L49" s="142"/>
+      <c r="M49" s="142"/>
+      <c r="N49" s="142"/>
+      <c r="O49" s="142"/>
+      <c r="P49" s="142"/>
+      <c r="Q49" s="85"/>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A50" s="84"/>
+      <c r="B50" s="142"/>
+      <c r="C50" s="142"/>
+      <c r="D50" s="142"/>
+      <c r="E50" s="142"/>
+      <c r="F50" s="85"/>
+      <c r="G50" s="84"/>
+      <c r="H50" s="142"/>
+      <c r="I50" s="142"/>
+      <c r="J50" s="142"/>
+      <c r="K50" s="142"/>
+      <c r="L50" s="142"/>
+      <c r="M50" s="142"/>
+      <c r="N50" s="142"/>
+      <c r="O50" s="142"/>
+      <c r="P50" s="142"/>
+      <c r="Q50" s="85"/>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A51" s="84"/>
+      <c r="B51" s="142"/>
+      <c r="C51" s="142"/>
+      <c r="D51" s="142"/>
+      <c r="E51" s="142"/>
+      <c r="F51" s="85"/>
+      <c r="G51" s="84"/>
+      <c r="H51" s="142"/>
+      <c r="I51" s="142"/>
+      <c r="J51" s="142"/>
+      <c r="K51" s="142"/>
+      <c r="L51" s="142"/>
+      <c r="M51" s="142"/>
+      <c r="N51" s="142"/>
+      <c r="O51" s="142"/>
+      <c r="P51" s="142"/>
+      <c r="Q51" s="85"/>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A52" s="84"/>
+      <c r="B52" s="142"/>
+      <c r="C52" s="142"/>
+      <c r="D52" s="142"/>
+      <c r="E52" s="142"/>
+      <c r="F52" s="85"/>
+      <c r="G52" s="84"/>
+      <c r="H52" s="142"/>
+      <c r="I52" s="142"/>
+      <c r="J52" s="142"/>
+      <c r="K52" s="142"/>
+      <c r="L52" s="142"/>
+      <c r="M52" s="142"/>
+      <c r="N52" s="142"/>
+      <c r="O52" s="142"/>
+      <c r="P52" s="142"/>
+      <c r="Q52" s="85"/>
+    </row>
+    <row r="53" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="86"/>
+      <c r="B53" s="44"/>
+      <c r="C53" s="44"/>
+      <c r="D53" s="44"/>
+      <c r="E53" s="44"/>
+      <c r="F53" s="87"/>
+      <c r="G53" s="86"/>
+      <c r="H53" s="44"/>
+      <c r="I53" s="44"/>
+      <c r="J53" s="44"/>
+      <c r="K53" s="44"/>
+      <c r="L53" s="44"/>
+      <c r="M53" s="44"/>
+      <c r="N53" s="44"/>
+      <c r="O53" s="44"/>
+      <c r="P53" s="44"/>
+      <c r="Q53" s="87"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F2"/>
+    <mergeCell ref="G1:Q2"/>
+  </mergeCells>
+  <phoneticPr fontId="14" type="noConversion"/>
+  <conditionalFormatting sqref="B4:B11">
+    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4786,133 +6096,175 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0E9D792-2517-4CE8-8D18-28421B01A876}">
-  <dimension ref="A2:N18"/>
+  <dimension ref="A2:N21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="48.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="54.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="30.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="132" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="108"/>
-      <c r="C2" s="108"/>
-      <c r="D2" s="108"/>
-      <c r="E2" s="108"/>
-      <c r="F2" s="108"/>
-    </row>
-    <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="82"/>
-      <c r="B4" s="83" t="s">
+      <c r="B2" s="132"/>
+      <c r="C2" s="132"/>
+      <c r="D2" s="132"/>
+      <c r="E2" s="132"/>
+      <c r="F2" s="132"/>
+    </row>
+    <row r="4" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:14" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="82"/>
+      <c r="B5" s="109" t="s">
+        <v>148</v>
+      </c>
+      <c r="H5" s="82"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="36"/>
+      <c r="M5" s="36"/>
+      <c r="N5" s="83"/>
+    </row>
+    <row r="6" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="84"/>
+      <c r="B6" s="83" t="s">
         <v>63</v>
       </c>
-      <c r="H4" s="82"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="83"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="84"/>
-      <c r="B5" s="85" t="s">
+      <c r="H6" s="84"/>
+      <c r="I6" s="142"/>
+      <c r="J6" s="142"/>
+      <c r="K6" s="142"/>
+      <c r="L6" s="142"/>
+      <c r="M6" s="142"/>
+      <c r="N6" s="85"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="84"/>
+      <c r="B7" s="85" t="s">
         <v>124</v>
       </c>
-      <c r="H5" s="84"/>
-      <c r="I5" s="108" t="s">
+      <c r="H7" s="84"/>
+      <c r="I7" s="132" t="s">
         <v>143</v>
       </c>
-      <c r="J5" s="108"/>
-      <c r="K5" s="108"/>
-      <c r="L5" s="108"/>
-      <c r="M5" s="108"/>
-      <c r="N5" s="109"/>
-    </row>
-    <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="86"/>
-      <c r="B6" s="87"/>
-      <c r="H6" s="84"/>
-      <c r="N6" s="85"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H7" s="84"/>
-      <c r="I7" t="s">
+      <c r="J7" s="132"/>
+      <c r="K7" s="132"/>
+      <c r="L7" s="132"/>
+      <c r="M7" s="132"/>
+      <c r="N7" s="133"/>
+    </row>
+    <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="86"/>
+      <c r="B8" s="87"/>
+      <c r="H8" s="84"/>
+      <c r="N8" s="85"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="142"/>
+      <c r="B9" s="142"/>
+      <c r="H9" s="84"/>
+      <c r="N9" s="85"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H10" s="84"/>
+      <c r="I10" t="s">
         <v>141</v>
       </c>
-      <c r="N7" s="85"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H8" s="84"/>
-      <c r="I8" t="s">
+      <c r="N10" s="85"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H11" s="84"/>
+      <c r="I11" t="s">
         <v>142</v>
       </c>
-      <c r="N8" s="85"/>
-    </row>
-    <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="H9" s="86"/>
-      <c r="I9" s="44"/>
-      <c r="J9" s="44"/>
-      <c r="K9" s="44"/>
-      <c r="L9" s="44"/>
-      <c r="M9" s="44"/>
-      <c r="N9" s="87"/>
-    </row>
-    <row r="10" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H11" s="82"/>
-      <c r="I11" s="36"/>
-      <c r="J11" s="36"/>
-      <c r="K11" s="36"/>
-      <c r="L11" s="83"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H12" s="84"/>
-      <c r="L12" s="85"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H13" s="84"/>
-      <c r="I13" s="110" t="s">
+      <c r="N11" s="85"/>
+    </row>
+    <row r="12" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H12" s="86"/>
+      <c r="I12" s="44"/>
+      <c r="J12" s="44"/>
+      <c r="K12" s="44"/>
+      <c r="L12" s="44"/>
+      <c r="M12" s="44"/>
+      <c r="N12" s="87"/>
+    </row>
+    <row r="13" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="82"/>
+      <c r="B13" s="109" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="84"/>
+      <c r="B14" s="85"/>
+      <c r="H14" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="I14" s="110" t="s">
+        <v>102</v>
+      </c>
+      <c r="J14" s="36"/>
+      <c r="K14" s="36"/>
+      <c r="L14" s="83"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="84"/>
+      <c r="B15" s="108" t="s">
+        <v>146</v>
+      </c>
+      <c r="H15" s="84"/>
+      <c r="L15" s="85"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="84"/>
+      <c r="B16" s="108" t="s">
+        <v>147</v>
+      </c>
+      <c r="H16" s="84"/>
+      <c r="I16" s="134" t="s">
         <v>145</v>
       </c>
-      <c r="J13" s="110"/>
-      <c r="K13" s="110"/>
-      <c r="L13" s="111"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H14" s="84"/>
-      <c r="L14" s="85"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H15" s="84"/>
-      <c r="I15" t="s">
-        <v>144</v>
-      </c>
-      <c r="L15" s="85"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H16" s="84"/>
-      <c r="L16" s="85"/>
-    </row>
-    <row r="17" spans="8:12" x14ac:dyDescent="0.25">
+      <c r="J16" s="134"/>
+      <c r="K16" s="134"/>
+      <c r="L16" s="135"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="84"/>
+      <c r="B17" s="85"/>
       <c r="H17" s="84"/>
       <c r="L17" s="85"/>
     </row>
-    <row r="18" spans="8:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="H18" s="86"/>
-      <c r="I18" s="44"/>
-      <c r="J18" s="44"/>
-      <c r="K18" s="44"/>
-      <c r="L18" s="87"/>
+    <row r="18" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="86"/>
+      <c r="B18" s="87"/>
+      <c r="H18" s="84"/>
+      <c r="I18" t="s">
+        <v>144</v>
+      </c>
+      <c r="L18" s="85"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H19" s="84"/>
+      <c r="L19" s="85"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H20" s="84"/>
+      <c r="L20" s="85"/>
+    </row>
+    <row r="21" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H21" s="86"/>
+      <c r="I21" s="44"/>
+      <c r="J21" s="44"/>
+      <c r="K21" s="44"/>
+      <c r="L21" s="87"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="I5:N5"/>
-    <mergeCell ref="I13:L13"/>
+    <mergeCell ref="I7:N7"/>
+    <mergeCell ref="I16:L16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>